<commit_message>
etl adjusted with new models replacing raw sql
</commit_message>
<xml_diff>
--- a/flask-backend/ETL/Fall 2025 Master Schedule - Copy.xlsx
+++ b/flask-backend/ETL/Fall 2025 Master Schedule - Copy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Domin\OneDrive - University of Nevada, Reno\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Domin\Desktop\senior_project\NCS_repo\flask-backend\ETL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77D5F596-EC2B-47FC-AC8E-F4AF2B27FF6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F23D3F26-4F65-44FE-9101-01E153607FCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4450" yWindow="2650" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>